<commit_message>
feat: add customer_retention heatmap
</commit_message>
<xml_diff>
--- a/analysis/excel/customer_retention.xlsx
+++ b/analysis/excel/customer_retention.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/DataGripProjects/olist-cohort-analysis/analysis/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF7B991E-5891-0D4F-9D5E-878FC6B7F8A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCF4E5C5-D955-A44D-8A86-C9E4845D8800}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="41020" xr2:uid="{FFB4930C-C763-C84A-B491-5777D21231B9}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="43760" windowHeight="41020" xr2:uid="{FFB4930C-C763-C84A-B491-5777D21231B9}"/>
   </bookViews>
   <sheets>
     <sheet name="retention_final" sheetId="20" r:id="rId1"/>
@@ -19,6 +19,9 @@
     <definedName name="ExternalData_1" localSheetId="0" hidden="1">'retention_final'!$A$1:$E$82</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
+  <pivotCaches>
+    <pivotCache cacheId="0" r:id="rId2"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -86,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>cohort_month</t>
   </si>
@@ -102,6 +105,15 @@
   <si>
     <t>retention_rate</t>
   </si>
+  <si>
+    <t>Average of retention_rate</t>
+  </si>
+  <si>
+    <t>Cohort Months</t>
+  </si>
+  <si>
+    <t>Months since first purchase</t>
+  </si>
 </sst>
 </file>
 
@@ -116,12 +128,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -136,16 +154,43 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yy"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0" tint="-0.34998626667073579"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -158,6 +203,1575 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Adam Czapla" refreshedDate="46136.677208796296" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="81" xr:uid="{64F79C19-8489-F448-9464-DC328CA485B4}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="retention_final"/>
+  </cacheSource>
+  <cacheFields count="7">
+    <cacheField name="cohort_month" numFmtId="14">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2017-01-01T00:00:00" maxDate="2017-09-02T00:00:00" count="9">
+        <d v="2017-01-01T00:00:00"/>
+        <d v="2017-02-01T00:00:00"/>
+        <d v="2017-03-01T00:00:00"/>
+        <d v="2017-04-01T00:00:00"/>
+        <d v="2017-05-01T00:00:00"/>
+        <d v="2017-06-01T00:00:00"/>
+        <d v="2017-07-01T00:00:00"/>
+        <d v="2017-08-01T00:00:00"/>
+        <d v="2017-09-01T00:00:00"/>
+      </sharedItems>
+      <fieldGroup par="6"/>
+    </cacheField>
+    <cacheField name="month_number" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="8" count="9">
+        <n v="0"/>
+        <n v="1"/>
+        <n v="2"/>
+        <n v="3"/>
+        <n v="4"/>
+        <n v="5"/>
+        <n v="6"/>
+        <n v="7"/>
+        <n v="8"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="active_customers" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="4057"/>
+    </cacheField>
+    <cacheField name="cohort_size" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="717" maxValue="4057"/>
+    </cacheField>
+    <cacheField name="retention_rate" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1.0660000000000001E-3" maxValue="1"/>
+    </cacheField>
+    <cacheField name="Days (cohort_month)" numFmtId="0" databaseField="0">
+      <fieldGroup base="0">
+        <rangePr groupBy="days" startDate="2017-01-01T00:00:00" endDate="2017-09-02T00:00:00"/>
+        <groupItems count="368">
+          <s v="&lt;01.01.17"/>
+          <s v="01. Jan"/>
+          <s v="02. Jan"/>
+          <s v="03. Jan"/>
+          <s v="04. Jan"/>
+          <s v="05. Jan"/>
+          <s v="06. Jan"/>
+          <s v="07. Jan"/>
+          <s v="08. Jan"/>
+          <s v="09. Jan"/>
+          <s v="10. Jan"/>
+          <s v="11. Jan"/>
+          <s v="12. Jan"/>
+          <s v="13. Jan"/>
+          <s v="14. Jan"/>
+          <s v="15. Jan"/>
+          <s v="16. Jan"/>
+          <s v="17. Jan"/>
+          <s v="18. Jan"/>
+          <s v="19. Jan"/>
+          <s v="20. Jan"/>
+          <s v="21. Jan"/>
+          <s v="22. Jan"/>
+          <s v="23. Jan"/>
+          <s v="24. Jan"/>
+          <s v="25. Jan"/>
+          <s v="26. Jan"/>
+          <s v="27. Jan"/>
+          <s v="28. Jan"/>
+          <s v="29. Jan"/>
+          <s v="30. Jan"/>
+          <s v="31. Jan"/>
+          <s v="01. Feb"/>
+          <s v="02. Feb"/>
+          <s v="03. Feb"/>
+          <s v="04. Feb"/>
+          <s v="05. Feb"/>
+          <s v="06. Feb"/>
+          <s v="07. Feb"/>
+          <s v="08. Feb"/>
+          <s v="09. Feb"/>
+          <s v="10. Feb"/>
+          <s v="11. Feb"/>
+          <s v="12. Feb"/>
+          <s v="13. Feb"/>
+          <s v="14. Feb"/>
+          <s v="15. Feb"/>
+          <s v="16. Feb"/>
+          <s v="17. Feb"/>
+          <s v="18. Feb"/>
+          <s v="19. Feb"/>
+          <s v="20. Feb"/>
+          <s v="21. Feb"/>
+          <s v="22. Feb"/>
+          <s v="23. Feb"/>
+          <s v="24. Feb"/>
+          <s v="25. Feb"/>
+          <s v="26. Feb"/>
+          <s v="27. Feb"/>
+          <s v="28. Feb"/>
+          <s v="29. Feb"/>
+          <s v="01. Mar"/>
+          <s v="02. Mar"/>
+          <s v="03. Mar"/>
+          <s v="04. Mar"/>
+          <s v="05. Mar"/>
+          <s v="06. Mar"/>
+          <s v="07. Mar"/>
+          <s v="08. Mar"/>
+          <s v="09. Mar"/>
+          <s v="10. Mar"/>
+          <s v="11. Mar"/>
+          <s v="12. Mar"/>
+          <s v="13. Mar"/>
+          <s v="14. Mar"/>
+          <s v="15. Mar"/>
+          <s v="16. Mar"/>
+          <s v="17. Mar"/>
+          <s v="18. Mar"/>
+          <s v="19. Mar"/>
+          <s v="20. Mar"/>
+          <s v="21. Mar"/>
+          <s v="22. Mar"/>
+          <s v="23. Mar"/>
+          <s v="24. Mar"/>
+          <s v="25. Mar"/>
+          <s v="26. Mar"/>
+          <s v="27. Mar"/>
+          <s v="28. Mar"/>
+          <s v="29. Mar"/>
+          <s v="30. Mar"/>
+          <s v="31. Mar"/>
+          <s v="01. Apr"/>
+          <s v="02. Apr"/>
+          <s v="03. Apr"/>
+          <s v="04. Apr"/>
+          <s v="05. Apr"/>
+          <s v="06. Apr"/>
+          <s v="07. Apr"/>
+          <s v="08. Apr"/>
+          <s v="09. Apr"/>
+          <s v="10. Apr"/>
+          <s v="11. Apr"/>
+          <s v="12. Apr"/>
+          <s v="13. Apr"/>
+          <s v="14. Apr"/>
+          <s v="15. Apr"/>
+          <s v="16. Apr"/>
+          <s v="17. Apr"/>
+          <s v="18. Apr"/>
+          <s v="19. Apr"/>
+          <s v="20. Apr"/>
+          <s v="21. Apr"/>
+          <s v="22. Apr"/>
+          <s v="23. Apr"/>
+          <s v="24. Apr"/>
+          <s v="25. Apr"/>
+          <s v="26. Apr"/>
+          <s v="27. Apr"/>
+          <s v="28. Apr"/>
+          <s v="29. Apr"/>
+          <s v="30. Apr"/>
+          <s v="01. May"/>
+          <s v="02. May"/>
+          <s v="03. May"/>
+          <s v="04. May"/>
+          <s v="05. May"/>
+          <s v="06. May"/>
+          <s v="07. May"/>
+          <s v="08. May"/>
+          <s v="09. May"/>
+          <s v="10. May"/>
+          <s v="11. May"/>
+          <s v="12. May"/>
+          <s v="13. May"/>
+          <s v="14. May"/>
+          <s v="15. May"/>
+          <s v="16. May"/>
+          <s v="17. May"/>
+          <s v="18. May"/>
+          <s v="19. May"/>
+          <s v="20. May"/>
+          <s v="21. May"/>
+          <s v="22. May"/>
+          <s v="23. May"/>
+          <s v="24. May"/>
+          <s v="25. May"/>
+          <s v="26. May"/>
+          <s v="27. May"/>
+          <s v="28. May"/>
+          <s v="29. May"/>
+          <s v="30. May"/>
+          <s v="31. May"/>
+          <s v="01. Jun"/>
+          <s v="02. Jun"/>
+          <s v="03. Jun"/>
+          <s v="04. Jun"/>
+          <s v="05. Jun"/>
+          <s v="06. Jun"/>
+          <s v="07. Jun"/>
+          <s v="08. Jun"/>
+          <s v="09. Jun"/>
+          <s v="10. Jun"/>
+          <s v="11. Jun"/>
+          <s v="12. Jun"/>
+          <s v="13. Jun"/>
+          <s v="14. Jun"/>
+          <s v="15. Jun"/>
+          <s v="16. Jun"/>
+          <s v="17. Jun"/>
+          <s v="18. Jun"/>
+          <s v="19. Jun"/>
+          <s v="20. Jun"/>
+          <s v="21. Jun"/>
+          <s v="22. Jun"/>
+          <s v="23. Jun"/>
+          <s v="24. Jun"/>
+          <s v="25. Jun"/>
+          <s v="26. Jun"/>
+          <s v="27. Jun"/>
+          <s v="28. Jun"/>
+          <s v="29. Jun"/>
+          <s v="30. Jun"/>
+          <s v="01. Jul"/>
+          <s v="02. Jul"/>
+          <s v="03. Jul"/>
+          <s v="04. Jul"/>
+          <s v="05. Jul"/>
+          <s v="06. Jul"/>
+          <s v="07. Jul"/>
+          <s v="08. Jul"/>
+          <s v="09. Jul"/>
+          <s v="10. Jul"/>
+          <s v="11. Jul"/>
+          <s v="12. Jul"/>
+          <s v="13. Jul"/>
+          <s v="14. Jul"/>
+          <s v="15. Jul"/>
+          <s v="16. Jul"/>
+          <s v="17. Jul"/>
+          <s v="18. Jul"/>
+          <s v="19. Jul"/>
+          <s v="20. Jul"/>
+          <s v="21. Jul"/>
+          <s v="22. Jul"/>
+          <s v="23. Jul"/>
+          <s v="24. Jul"/>
+          <s v="25. Jul"/>
+          <s v="26. Jul"/>
+          <s v="27. Jul"/>
+          <s v="28. Jul"/>
+          <s v="29. Jul"/>
+          <s v="30. Jul"/>
+          <s v="31. Jul"/>
+          <s v="01. Aug"/>
+          <s v="02. Aug"/>
+          <s v="03. Aug"/>
+          <s v="04. Aug"/>
+          <s v="05. Aug"/>
+          <s v="06. Aug"/>
+          <s v="07. Aug"/>
+          <s v="08. Aug"/>
+          <s v="09. Aug"/>
+          <s v="10. Aug"/>
+          <s v="11. Aug"/>
+          <s v="12. Aug"/>
+          <s v="13. Aug"/>
+          <s v="14. Aug"/>
+          <s v="15. Aug"/>
+          <s v="16. Aug"/>
+          <s v="17. Aug"/>
+          <s v="18. Aug"/>
+          <s v="19. Aug"/>
+          <s v="20. Aug"/>
+          <s v="21. Aug"/>
+          <s v="22. Aug"/>
+          <s v="23. Aug"/>
+          <s v="24. Aug"/>
+          <s v="25. Aug"/>
+          <s v="26. Aug"/>
+          <s v="27. Aug"/>
+          <s v="28. Aug"/>
+          <s v="29. Aug"/>
+          <s v="30. Aug"/>
+          <s v="31. Aug"/>
+          <s v="01. Sep"/>
+          <s v="02. Sep"/>
+          <s v="03. Sep"/>
+          <s v="04. Sep"/>
+          <s v="05. Sep"/>
+          <s v="06. Sep"/>
+          <s v="07. Sep"/>
+          <s v="08. Sep"/>
+          <s v="09. Sep"/>
+          <s v="10. Sep"/>
+          <s v="11. Sep"/>
+          <s v="12. Sep"/>
+          <s v="13. Sep"/>
+          <s v="14. Sep"/>
+          <s v="15. Sep"/>
+          <s v="16. Sep"/>
+          <s v="17. Sep"/>
+          <s v="18. Sep"/>
+          <s v="19. Sep"/>
+          <s v="20. Sep"/>
+          <s v="21. Sep"/>
+          <s v="22. Sep"/>
+          <s v="23. Sep"/>
+          <s v="24. Sep"/>
+          <s v="25. Sep"/>
+          <s v="26. Sep"/>
+          <s v="27. Sep"/>
+          <s v="28. Sep"/>
+          <s v="29. Sep"/>
+          <s v="30. Sep"/>
+          <s v="01. Oct"/>
+          <s v="02. Oct"/>
+          <s v="03. Oct"/>
+          <s v="04. Oct"/>
+          <s v="05. Oct"/>
+          <s v="06. Oct"/>
+          <s v="07. Oct"/>
+          <s v="08. Oct"/>
+          <s v="09. Oct"/>
+          <s v="10. Oct"/>
+          <s v="11. Oct"/>
+          <s v="12. Oct"/>
+          <s v="13. Oct"/>
+          <s v="14. Oct"/>
+          <s v="15. Oct"/>
+          <s v="16. Oct"/>
+          <s v="17. Oct"/>
+          <s v="18. Oct"/>
+          <s v="19. Oct"/>
+          <s v="20. Oct"/>
+          <s v="21. Oct"/>
+          <s v="22. Oct"/>
+          <s v="23. Oct"/>
+          <s v="24. Oct"/>
+          <s v="25. Oct"/>
+          <s v="26. Oct"/>
+          <s v="27. Oct"/>
+          <s v="28. Oct"/>
+          <s v="29. Oct"/>
+          <s v="30. Oct"/>
+          <s v="31. Oct"/>
+          <s v="01. Nov"/>
+          <s v="02. Nov"/>
+          <s v="03. Nov"/>
+          <s v="04. Nov"/>
+          <s v="05. Nov"/>
+          <s v="06. Nov"/>
+          <s v="07. Nov"/>
+          <s v="08. Nov"/>
+          <s v="09. Nov"/>
+          <s v="10. Nov"/>
+          <s v="11. Nov"/>
+          <s v="12. Nov"/>
+          <s v="13. Nov"/>
+          <s v="14. Nov"/>
+          <s v="15. Nov"/>
+          <s v="16. Nov"/>
+          <s v="17. Nov"/>
+          <s v="18. Nov"/>
+          <s v="19. Nov"/>
+          <s v="20. Nov"/>
+          <s v="21. Nov"/>
+          <s v="22. Nov"/>
+          <s v="23. Nov"/>
+          <s v="24. Nov"/>
+          <s v="25. Nov"/>
+          <s v="26. Nov"/>
+          <s v="27. Nov"/>
+          <s v="28. Nov"/>
+          <s v="29. Nov"/>
+          <s v="30. Nov"/>
+          <s v="01. Dec"/>
+          <s v="02. Dec"/>
+          <s v="03. Dec"/>
+          <s v="04. Dec"/>
+          <s v="05. Dec"/>
+          <s v="06. Dec"/>
+          <s v="07. Dec"/>
+          <s v="08. Dec"/>
+          <s v="09. Dec"/>
+          <s v="10. Dec"/>
+          <s v="11. Dec"/>
+          <s v="12. Dec"/>
+          <s v="13. Dec"/>
+          <s v="14. Dec"/>
+          <s v="15. Dec"/>
+          <s v="16. Dec"/>
+          <s v="17. Dec"/>
+          <s v="18. Dec"/>
+          <s v="19. Dec"/>
+          <s v="20. Dec"/>
+          <s v="21. Dec"/>
+          <s v="22. Dec"/>
+          <s v="23. Dec"/>
+          <s v="24. Dec"/>
+          <s v="25. Dec"/>
+          <s v="26. Dec"/>
+          <s v="27. Dec"/>
+          <s v="28. Dec"/>
+          <s v="29. Dec"/>
+          <s v="30. Dec"/>
+          <s v="31. Dec"/>
+          <s v="&gt;02.09.17"/>
+        </groupItems>
+      </fieldGroup>
+    </cacheField>
+    <cacheField name="Months (cohort_month)" numFmtId="0" databaseField="0">
+      <fieldGroup base="0">
+        <rangePr groupBy="months" startDate="2017-01-01T00:00:00" endDate="2017-09-02T00:00:00"/>
+        <groupItems count="14">
+          <s v="&lt;01.01.17"/>
+          <s v="Jan"/>
+          <s v="Feb"/>
+          <s v="Mar"/>
+          <s v="Apr"/>
+          <s v="May"/>
+          <s v="Jun"/>
+          <s v="Jul"/>
+          <s v="Aug"/>
+          <s v="Sep"/>
+          <s v="Oct"/>
+          <s v="Nov"/>
+          <s v="Dec"/>
+          <s v="&gt;02.09.17"/>
+        </groupItems>
+      </fieldGroup>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="81">
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="717"/>
+    <n v="717"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="1"/>
+    <n v="2"/>
+    <n v="717"/>
+    <n v="2.7889999999999998E-3"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="2"/>
+    <n v="2"/>
+    <n v="717"/>
+    <n v="2.7889999999999998E-3"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="3"/>
+    <n v="1"/>
+    <n v="717"/>
+    <n v="1.395E-3"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="4"/>
+    <n v="3"/>
+    <n v="717"/>
+    <n v="4.1840000000000002E-3"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="5"/>
+    <n v="1"/>
+    <n v="717"/>
+    <n v="1.395E-3"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="6"/>
+    <n v="3"/>
+    <n v="717"/>
+    <n v="4.1840000000000002E-3"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="7"/>
+    <n v="1"/>
+    <n v="717"/>
+    <n v="1.395E-3"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="8"/>
+    <n v="1"/>
+    <n v="717"/>
+    <n v="1.395E-3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="1628"/>
+    <n v="1628"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="3"/>
+    <n v="1628"/>
+    <n v="1.843E-3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="2"/>
+    <n v="5"/>
+    <n v="1628"/>
+    <n v="3.0709999999999999E-3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="3"/>
+    <n v="2"/>
+    <n v="1628"/>
+    <n v="1.2290000000000001E-3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="4"/>
+    <n v="7"/>
+    <n v="1628"/>
+    <n v="4.3E-3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="5"/>
+    <n v="2"/>
+    <n v="1628"/>
+    <n v="1.2290000000000001E-3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="6"/>
+    <n v="4"/>
+    <n v="1628"/>
+    <n v="2.457E-3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="7"/>
+    <n v="3"/>
+    <n v="1628"/>
+    <n v="1.843E-3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="8"/>
+    <n v="2"/>
+    <n v="1628"/>
+    <n v="1.2290000000000001E-3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="2503"/>
+    <n v="2503"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="1"/>
+    <n v="11"/>
+    <n v="2503"/>
+    <n v="4.3949999999999996E-3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <n v="9"/>
+    <n v="2503"/>
+    <n v="3.5959999999999998E-3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="3"/>
+    <n v="10"/>
+    <n v="2503"/>
+    <n v="3.9950000000000003E-3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="4"/>
+    <n v="9"/>
+    <n v="2503"/>
+    <n v="3.5959999999999998E-3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="5"/>
+    <n v="4"/>
+    <n v="2503"/>
+    <n v="1.598E-3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="6"/>
+    <n v="4"/>
+    <n v="2503"/>
+    <n v="1.598E-3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="7"/>
+    <n v="8"/>
+    <n v="2503"/>
+    <n v="3.1960000000000001E-3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="8"/>
+    <n v="8"/>
+    <n v="2503"/>
+    <n v="3.1960000000000001E-3"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="2256"/>
+    <n v="2256"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="1"/>
+    <n v="14"/>
+    <n v="2256"/>
+    <n v="6.2059999999999997E-3"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="2"/>
+    <n v="5"/>
+    <n v="2256"/>
+    <n v="2.2160000000000001E-3"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="3"/>
+    <n v="4"/>
+    <n v="2256"/>
+    <n v="1.7730000000000001E-3"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="4"/>
+    <n v="6"/>
+    <n v="2256"/>
+    <n v="2.66E-3"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="5"/>
+    <n v="6"/>
+    <n v="2256"/>
+    <n v="2.66E-3"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="6"/>
+    <n v="8"/>
+    <n v="2256"/>
+    <n v="3.5460000000000001E-3"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="7"/>
+    <n v="7"/>
+    <n v="2256"/>
+    <n v="3.1029999999999999E-3"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="8"/>
+    <n v="7"/>
+    <n v="2256"/>
+    <n v="3.1029999999999999E-3"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="0"/>
+    <n v="3451"/>
+    <n v="3451"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="1"/>
+    <n v="16"/>
+    <n v="3451"/>
+    <n v="4.6360000000000004E-3"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="2"/>
+    <n v="16"/>
+    <n v="3451"/>
+    <n v="4.6360000000000004E-3"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="3"/>
+    <n v="10"/>
+    <n v="3451"/>
+    <n v="2.898E-3"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="4"/>
+    <n v="10"/>
+    <n v="3451"/>
+    <n v="2.898E-3"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="5"/>
+    <n v="11"/>
+    <n v="3451"/>
+    <n v="3.1870000000000002E-3"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="6"/>
+    <n v="14"/>
+    <n v="3451"/>
+    <n v="4.0569999999999998E-3"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="7"/>
+    <n v="5"/>
+    <n v="3451"/>
+    <n v="1.449E-3"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="8"/>
+    <n v="9"/>
+    <n v="3451"/>
+    <n v="2.6080000000000001E-3"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="0"/>
+    <n v="3037"/>
+    <n v="3037"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="1"/>
+    <n v="15"/>
+    <n v="3037"/>
+    <n v="4.9389999999999998E-3"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="2"/>
+    <n v="12"/>
+    <n v="3037"/>
+    <n v="3.9509999999999997E-3"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="3"/>
+    <n v="13"/>
+    <n v="3037"/>
+    <n v="4.2810000000000001E-3"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="4"/>
+    <n v="9"/>
+    <n v="3037"/>
+    <n v="2.9629999999999999E-3"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="5"/>
+    <n v="12"/>
+    <n v="3037"/>
+    <n v="3.9509999999999997E-3"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="6"/>
+    <n v="11"/>
+    <n v="3037"/>
+    <n v="3.6219999999999998E-3"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="7"/>
+    <n v="7"/>
+    <n v="3037"/>
+    <n v="2.3050000000000002E-3"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="8"/>
+    <n v="4"/>
+    <n v="3037"/>
+    <n v="1.317E-3"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <x v="0"/>
+    <n v="3752"/>
+    <n v="3752"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <x v="1"/>
+    <n v="20"/>
+    <n v="3752"/>
+    <n v="5.3299999999999997E-3"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <x v="2"/>
+    <n v="13"/>
+    <n v="3752"/>
+    <n v="3.4650000000000002E-3"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <x v="3"/>
+    <n v="9"/>
+    <n v="3752"/>
+    <n v="2.3990000000000001E-3"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <x v="4"/>
+    <n v="11"/>
+    <n v="3752"/>
+    <n v="2.9320000000000001E-3"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <x v="5"/>
+    <n v="8"/>
+    <n v="3752"/>
+    <n v="2.1320000000000002E-3"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <x v="6"/>
+    <n v="12"/>
+    <n v="3752"/>
+    <n v="3.1979999999999999E-3"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <x v="7"/>
+    <n v="4"/>
+    <n v="3752"/>
+    <n v="1.0660000000000001E-3"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <x v="8"/>
+    <n v="7"/>
+    <n v="3752"/>
+    <n v="1.866E-3"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <x v="0"/>
+    <n v="4057"/>
+    <n v="4057"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <x v="1"/>
+    <n v="28"/>
+    <n v="4057"/>
+    <n v="6.9020000000000001E-3"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <x v="2"/>
+    <n v="14"/>
+    <n v="4057"/>
+    <n v="3.4510000000000001E-3"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <x v="3"/>
+    <n v="11"/>
+    <n v="4057"/>
+    <n v="2.7109999999999999E-3"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <x v="4"/>
+    <n v="14"/>
+    <n v="4057"/>
+    <n v="3.4510000000000001E-3"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <x v="5"/>
+    <n v="21"/>
+    <n v="4057"/>
+    <n v="5.176E-3"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <x v="6"/>
+    <n v="12"/>
+    <n v="4057"/>
+    <n v="2.9580000000000001E-3"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <x v="7"/>
+    <n v="11"/>
+    <n v="4057"/>
+    <n v="2.7109999999999999E-3"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <x v="8"/>
+    <n v="6"/>
+    <n v="4057"/>
+    <n v="1.4790000000000001E-3"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="0"/>
+    <n v="4004"/>
+    <n v="4004"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="1"/>
+    <n v="28"/>
+    <n v="4004"/>
+    <n v="6.9930000000000001E-3"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="2"/>
+    <n v="22"/>
+    <n v="4004"/>
+    <n v="5.4949999999999999E-3"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="3"/>
+    <n v="11"/>
+    <n v="4004"/>
+    <n v="2.7469999999999999E-3"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="4"/>
+    <n v="18"/>
+    <n v="4004"/>
+    <n v="4.496E-3"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="5"/>
+    <n v="9"/>
+    <n v="4004"/>
+    <n v="2.248E-3"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="6"/>
+    <n v="9"/>
+    <n v="4004"/>
+    <n v="2.248E-3"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="7"/>
+    <n v="10"/>
+    <n v="4004"/>
+    <n v="2.4979999999999998E-3"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="8"/>
+    <n v="11"/>
+    <n v="4004"/>
+    <n v="2.7469999999999999E-3"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{69B9DD8B-EFE9-A444-97D9-43AE4E925D8A}" name="customer_retention" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Cohort Months" colHeaderCaption="Months since first purchase">
+  <location ref="G1:P11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="7">
+    <pivotField axis="axisRow" numFmtId="14" showAll="0">
+      <items count="10">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="10">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="369">
+        <item sd="0" x="0"/>
+        <item x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+        <item sd="0" x="6"/>
+        <item sd="0" x="7"/>
+        <item sd="0" x="8"/>
+        <item sd="0" x="9"/>
+        <item sd="0" x="10"/>
+        <item sd="0" x="11"/>
+        <item sd="0" x="12"/>
+        <item sd="0" x="13"/>
+        <item sd="0" x="14"/>
+        <item sd="0" x="15"/>
+        <item sd="0" x="16"/>
+        <item sd="0" x="17"/>
+        <item sd="0" x="18"/>
+        <item sd="0" x="19"/>
+        <item sd="0" x="20"/>
+        <item sd="0" x="21"/>
+        <item sd="0" x="22"/>
+        <item sd="0" x="23"/>
+        <item sd="0" x="24"/>
+        <item sd="0" x="25"/>
+        <item sd="0" x="26"/>
+        <item sd="0" x="27"/>
+        <item sd="0" x="28"/>
+        <item sd="0" x="29"/>
+        <item sd="0" x="30"/>
+        <item sd="0" x="31"/>
+        <item sd="0" x="32"/>
+        <item sd="0" x="33"/>
+        <item sd="0" x="34"/>
+        <item sd="0" x="35"/>
+        <item sd="0" x="36"/>
+        <item sd="0" x="37"/>
+        <item sd="0" x="38"/>
+        <item sd="0" x="39"/>
+        <item sd="0" x="40"/>
+        <item sd="0" x="41"/>
+        <item sd="0" x="42"/>
+        <item sd="0" x="43"/>
+        <item sd="0" x="44"/>
+        <item sd="0" x="45"/>
+        <item sd="0" x="46"/>
+        <item sd="0" x="47"/>
+        <item sd="0" x="48"/>
+        <item sd="0" x="49"/>
+        <item sd="0" x="50"/>
+        <item sd="0" x="51"/>
+        <item sd="0" x="52"/>
+        <item sd="0" x="53"/>
+        <item sd="0" x="54"/>
+        <item sd="0" x="55"/>
+        <item sd="0" x="56"/>
+        <item sd="0" x="57"/>
+        <item sd="0" x="58"/>
+        <item sd="0" x="59"/>
+        <item sd="0" x="60"/>
+        <item sd="0" x="61"/>
+        <item sd="0" x="62"/>
+        <item sd="0" x="63"/>
+        <item sd="0" x="64"/>
+        <item sd="0" x="65"/>
+        <item sd="0" x="66"/>
+        <item sd="0" x="67"/>
+        <item sd="0" x="68"/>
+        <item sd="0" x="69"/>
+        <item sd="0" x="70"/>
+        <item sd="0" x="71"/>
+        <item sd="0" x="72"/>
+        <item sd="0" x="73"/>
+        <item sd="0" x="74"/>
+        <item sd="0" x="75"/>
+        <item sd="0" x="76"/>
+        <item sd="0" x="77"/>
+        <item sd="0" x="78"/>
+        <item sd="0" x="79"/>
+        <item sd="0" x="80"/>
+        <item sd="0" x="81"/>
+        <item sd="0" x="82"/>
+        <item sd="0" x="83"/>
+        <item sd="0" x="84"/>
+        <item sd="0" x="85"/>
+        <item sd="0" x="86"/>
+        <item sd="0" x="87"/>
+        <item sd="0" x="88"/>
+        <item sd="0" x="89"/>
+        <item sd="0" x="90"/>
+        <item sd="0" x="91"/>
+        <item sd="0" x="92"/>
+        <item sd="0" x="93"/>
+        <item sd="0" x="94"/>
+        <item sd="0" x="95"/>
+        <item sd="0" x="96"/>
+        <item sd="0" x="97"/>
+        <item sd="0" x="98"/>
+        <item sd="0" x="99"/>
+        <item sd="0" x="100"/>
+        <item sd="0" x="101"/>
+        <item sd="0" x="102"/>
+        <item sd="0" x="103"/>
+        <item sd="0" x="104"/>
+        <item sd="0" x="105"/>
+        <item sd="0" x="106"/>
+        <item sd="0" x="107"/>
+        <item sd="0" x="108"/>
+        <item sd="0" x="109"/>
+        <item sd="0" x="110"/>
+        <item sd="0" x="111"/>
+        <item sd="0" x="112"/>
+        <item sd="0" x="113"/>
+        <item sd="0" x="114"/>
+        <item sd="0" x="115"/>
+        <item sd="0" x="116"/>
+        <item sd="0" x="117"/>
+        <item sd="0" x="118"/>
+        <item sd="0" x="119"/>
+        <item sd="0" x="120"/>
+        <item sd="0" x="121"/>
+        <item sd="0" x="122"/>
+        <item sd="0" x="123"/>
+        <item sd="0" x="124"/>
+        <item sd="0" x="125"/>
+        <item sd="0" x="126"/>
+        <item sd="0" x="127"/>
+        <item sd="0" x="128"/>
+        <item sd="0" x="129"/>
+        <item sd="0" x="130"/>
+        <item sd="0" x="131"/>
+        <item sd="0" x="132"/>
+        <item sd="0" x="133"/>
+        <item sd="0" x="134"/>
+        <item sd="0" x="135"/>
+        <item sd="0" x="136"/>
+        <item sd="0" x="137"/>
+        <item sd="0" x="138"/>
+        <item sd="0" x="139"/>
+        <item sd="0" x="140"/>
+        <item sd="0" x="141"/>
+        <item sd="0" x="142"/>
+        <item sd="0" x="143"/>
+        <item sd="0" x="144"/>
+        <item sd="0" x="145"/>
+        <item sd="0" x="146"/>
+        <item sd="0" x="147"/>
+        <item sd="0" x="148"/>
+        <item sd="0" x="149"/>
+        <item sd="0" x="150"/>
+        <item sd="0" x="151"/>
+        <item sd="0" x="152"/>
+        <item sd="0" x="153"/>
+        <item sd="0" x="154"/>
+        <item sd="0" x="155"/>
+        <item sd="0" x="156"/>
+        <item sd="0" x="157"/>
+        <item sd="0" x="158"/>
+        <item sd="0" x="159"/>
+        <item sd="0" x="160"/>
+        <item sd="0" x="161"/>
+        <item sd="0" x="162"/>
+        <item sd="0" x="163"/>
+        <item sd="0" x="164"/>
+        <item sd="0" x="165"/>
+        <item sd="0" x="166"/>
+        <item sd="0" x="167"/>
+        <item sd="0" x="168"/>
+        <item sd="0" x="169"/>
+        <item sd="0" x="170"/>
+        <item sd="0" x="171"/>
+        <item sd="0" x="172"/>
+        <item sd="0" x="173"/>
+        <item sd="0" x="174"/>
+        <item sd="0" x="175"/>
+        <item sd="0" x="176"/>
+        <item sd="0" x="177"/>
+        <item sd="0" x="178"/>
+        <item sd="0" x="179"/>
+        <item sd="0" x="180"/>
+        <item sd="0" x="181"/>
+        <item sd="0" x="182"/>
+        <item sd="0" x="183"/>
+        <item sd="0" x="184"/>
+        <item sd="0" x="185"/>
+        <item sd="0" x="186"/>
+        <item sd="0" x="187"/>
+        <item sd="0" x="188"/>
+        <item sd="0" x="189"/>
+        <item sd="0" x="190"/>
+        <item sd="0" x="191"/>
+        <item sd="0" x="192"/>
+        <item sd="0" x="193"/>
+        <item sd="0" x="194"/>
+        <item sd="0" x="195"/>
+        <item sd="0" x="196"/>
+        <item sd="0" x="197"/>
+        <item sd="0" x="198"/>
+        <item sd="0" x="199"/>
+        <item sd="0" x="200"/>
+        <item sd="0" x="201"/>
+        <item sd="0" x="202"/>
+        <item sd="0" x="203"/>
+        <item sd="0" x="204"/>
+        <item sd="0" x="205"/>
+        <item sd="0" x="206"/>
+        <item sd="0" x="207"/>
+        <item sd="0" x="208"/>
+        <item sd="0" x="209"/>
+        <item sd="0" x="210"/>
+        <item sd="0" x="211"/>
+        <item sd="0" x="212"/>
+        <item sd="0" x="213"/>
+        <item sd="0" x="214"/>
+        <item sd="0" x="215"/>
+        <item sd="0" x="216"/>
+        <item sd="0" x="217"/>
+        <item sd="0" x="218"/>
+        <item sd="0" x="219"/>
+        <item sd="0" x="220"/>
+        <item sd="0" x="221"/>
+        <item sd="0" x="222"/>
+        <item sd="0" x="223"/>
+        <item sd="0" x="224"/>
+        <item sd="0" x="225"/>
+        <item sd="0" x="226"/>
+        <item sd="0" x="227"/>
+        <item sd="0" x="228"/>
+        <item sd="0" x="229"/>
+        <item sd="0" x="230"/>
+        <item sd="0" x="231"/>
+        <item sd="0" x="232"/>
+        <item sd="0" x="233"/>
+        <item sd="0" x="234"/>
+        <item sd="0" x="235"/>
+        <item sd="0" x="236"/>
+        <item sd="0" x="237"/>
+        <item sd="0" x="238"/>
+        <item sd="0" x="239"/>
+        <item sd="0" x="240"/>
+        <item sd="0" x="241"/>
+        <item sd="0" x="242"/>
+        <item sd="0" x="243"/>
+        <item sd="0" x="244"/>
+        <item sd="0" x="245"/>
+        <item sd="0" x="246"/>
+        <item sd="0" x="247"/>
+        <item sd="0" x="248"/>
+        <item sd="0" x="249"/>
+        <item sd="0" x="250"/>
+        <item sd="0" x="251"/>
+        <item sd="0" x="252"/>
+        <item sd="0" x="253"/>
+        <item sd="0" x="254"/>
+        <item sd="0" x="255"/>
+        <item sd="0" x="256"/>
+        <item sd="0" x="257"/>
+        <item sd="0" x="258"/>
+        <item sd="0" x="259"/>
+        <item sd="0" x="260"/>
+        <item sd="0" x="261"/>
+        <item sd="0" x="262"/>
+        <item sd="0" x="263"/>
+        <item sd="0" x="264"/>
+        <item sd="0" x="265"/>
+        <item sd="0" x="266"/>
+        <item sd="0" x="267"/>
+        <item sd="0" x="268"/>
+        <item sd="0" x="269"/>
+        <item sd="0" x="270"/>
+        <item sd="0" x="271"/>
+        <item sd="0" x="272"/>
+        <item sd="0" x="273"/>
+        <item sd="0" x="274"/>
+        <item sd="0" x="275"/>
+        <item sd="0" x="276"/>
+        <item sd="0" x="277"/>
+        <item sd="0" x="278"/>
+        <item sd="0" x="279"/>
+        <item sd="0" x="280"/>
+        <item sd="0" x="281"/>
+        <item sd="0" x="282"/>
+        <item sd="0" x="283"/>
+        <item sd="0" x="284"/>
+        <item sd="0" x="285"/>
+        <item sd="0" x="286"/>
+        <item sd="0" x="287"/>
+        <item sd="0" x="288"/>
+        <item sd="0" x="289"/>
+        <item sd="0" x="290"/>
+        <item sd="0" x="291"/>
+        <item sd="0" x="292"/>
+        <item sd="0" x="293"/>
+        <item sd="0" x="294"/>
+        <item sd="0" x="295"/>
+        <item sd="0" x="296"/>
+        <item sd="0" x="297"/>
+        <item sd="0" x="298"/>
+        <item sd="0" x="299"/>
+        <item sd="0" x="300"/>
+        <item sd="0" x="301"/>
+        <item sd="0" x="302"/>
+        <item sd="0" x="303"/>
+        <item sd="0" x="304"/>
+        <item sd="0" x="305"/>
+        <item sd="0" x="306"/>
+        <item sd="0" x="307"/>
+        <item sd="0" x="308"/>
+        <item sd="0" x="309"/>
+        <item sd="0" x="310"/>
+        <item sd="0" x="311"/>
+        <item sd="0" x="312"/>
+        <item sd="0" x="313"/>
+        <item sd="0" x="314"/>
+        <item sd="0" x="315"/>
+        <item sd="0" x="316"/>
+        <item sd="0" x="317"/>
+        <item sd="0" x="318"/>
+        <item sd="0" x="319"/>
+        <item sd="0" x="320"/>
+        <item sd="0" x="321"/>
+        <item sd="0" x="322"/>
+        <item sd="0" x="323"/>
+        <item sd="0" x="324"/>
+        <item sd="0" x="325"/>
+        <item sd="0" x="326"/>
+        <item sd="0" x="327"/>
+        <item sd="0" x="328"/>
+        <item sd="0" x="329"/>
+        <item sd="0" x="330"/>
+        <item sd="0" x="331"/>
+        <item sd="0" x="332"/>
+        <item sd="0" x="333"/>
+        <item sd="0" x="334"/>
+        <item sd="0" x="335"/>
+        <item sd="0" x="336"/>
+        <item sd="0" x="337"/>
+        <item sd="0" x="338"/>
+        <item sd="0" x="339"/>
+        <item sd="0" x="340"/>
+        <item sd="0" x="341"/>
+        <item sd="0" x="342"/>
+        <item sd="0" x="343"/>
+        <item sd="0" x="344"/>
+        <item sd="0" x="345"/>
+        <item sd="0" x="346"/>
+        <item sd="0" x="347"/>
+        <item sd="0" x="348"/>
+        <item sd="0" x="349"/>
+        <item sd="0" x="350"/>
+        <item sd="0" x="351"/>
+        <item sd="0" x="352"/>
+        <item sd="0" x="353"/>
+        <item sd="0" x="354"/>
+        <item sd="0" x="355"/>
+        <item sd="0" x="356"/>
+        <item sd="0" x="357"/>
+        <item sd="0" x="358"/>
+        <item sd="0" x="359"/>
+        <item sd="0" x="360"/>
+        <item sd="0" x="361"/>
+        <item sd="0" x="362"/>
+        <item sd="0" x="363"/>
+        <item sd="0" x="364"/>
+        <item sd="0" x="365"/>
+        <item sd="0" x="366"/>
+        <item sd="0" x="367"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="15">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+        <item sd="0" x="6"/>
+        <item sd="0" x="7"/>
+        <item sd="0" x="8"/>
+        <item sd="0" x="9"/>
+        <item sd="0" x="10"/>
+        <item sd="0" x="11"/>
+        <item sd="0" x="12"/>
+        <item sd="0" x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="9">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="9">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of retention_rate" fld="4" subtotal="average" baseField="0" baseItem="0" numFmtId="10"/>
+  </dataFields>
+  <formats count="2">
+    <format dxfId="3">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <conditionalFormats count="1">
+    <conditionalFormat priority="1">
+      <pivotAreas count="1">
+        <pivotArea type="data" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="1" count="8" selected="0">
+              <x v="1"/>
+              <x v="2"/>
+              <x v="3"/>
+              <x v="4"/>
+              <x v="5"/>
+              <x v="6"/>
+              <x v="7"/>
+              <x v="8"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </pivotAreas>
+    </conditionalFormat>
+  </conditionalFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -178,7 +1792,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B07A68E4-C711-0747-A693-1E26940D860C}" name="retention_final" displayName="retention_final" ref="A1:E82" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E82" xr:uid="{B07A68E4-C711-0747-A693-1E26940D860C}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{C1CD0E24-7A54-B947-AB45-4F2ABF7ECCF0}" uniqueName="1" name="cohort_month" queryTableFieldId="1" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{C1CD0E24-7A54-B947-AB45-4F2ABF7ECCF0}" uniqueName="1" name="cohort_month" queryTableFieldId="1" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{80426A89-325F-F041-B37C-376B9EA9B271}" uniqueName="2" name="month_number" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{F2B16E17-9653-244B-A26B-B332A4245277}" uniqueName="3" name="active_customers" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{65707286-E6B5-124F-87B4-94E2B7DCAC1E}" uniqueName="4" name="cohort_size" queryTableFieldId="4"/>
@@ -505,7 +2119,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF6A6796-3256-514F-8784-774FE4E6B314}">
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:P82"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.1640625" bestFit="1" customWidth="1"/>
@@ -513,9 +2127,13 @@
     <col min="3" max="3" width="18.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="16" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -531,8 +2149,14 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>42736</v>
       </c>
@@ -548,8 +2172,38 @@
       <c r="E2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>3</v>
+      </c>
+      <c r="L2">
+        <v>4</v>
+      </c>
+      <c r="M2">
+        <v>5</v>
+      </c>
+      <c r="N2">
+        <v>6</v>
+      </c>
+      <c r="O2">
+        <v>7</v>
+      </c>
+      <c r="P2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>42736</v>
       </c>
@@ -565,8 +2219,38 @@
       <c r="E3">
         <v>2.7889999999999998E-3</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G3" s="3">
+        <v>42736</v>
+      </c>
+      <c r="H3" s="5">
+        <v>1</v>
+      </c>
+      <c r="I3" s="4">
+        <v>2.7889999999999998E-3</v>
+      </c>
+      <c r="J3" s="4">
+        <v>2.7889999999999998E-3</v>
+      </c>
+      <c r="K3" s="4">
+        <v>1.395E-3</v>
+      </c>
+      <c r="L3" s="4">
+        <v>4.1840000000000002E-3</v>
+      </c>
+      <c r="M3" s="4">
+        <v>1.395E-3</v>
+      </c>
+      <c r="N3" s="4">
+        <v>4.1840000000000002E-3</v>
+      </c>
+      <c r="O3" s="4">
+        <v>1.395E-3</v>
+      </c>
+      <c r="P3" s="4">
+        <v>1.395E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>42736</v>
       </c>
@@ -582,8 +2266,38 @@
       <c r="E4">
         <v>2.7889999999999998E-3</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G4" s="3">
+        <v>42767</v>
+      </c>
+      <c r="H4" s="5">
+        <v>1</v>
+      </c>
+      <c r="I4" s="4">
+        <v>1.843E-3</v>
+      </c>
+      <c r="J4" s="4">
+        <v>3.0709999999999999E-3</v>
+      </c>
+      <c r="K4" s="4">
+        <v>1.2290000000000001E-3</v>
+      </c>
+      <c r="L4" s="4">
+        <v>4.3E-3</v>
+      </c>
+      <c r="M4" s="4">
+        <v>1.2290000000000001E-3</v>
+      </c>
+      <c r="N4" s="4">
+        <v>2.457E-3</v>
+      </c>
+      <c r="O4" s="4">
+        <v>1.843E-3</v>
+      </c>
+      <c r="P4" s="4">
+        <v>1.2290000000000001E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>42736</v>
       </c>
@@ -599,8 +2313,38 @@
       <c r="E5">
         <v>1.395E-3</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G5" s="3">
+        <v>42795</v>
+      </c>
+      <c r="H5" s="5">
+        <v>1</v>
+      </c>
+      <c r="I5" s="4">
+        <v>4.3949999999999996E-3</v>
+      </c>
+      <c r="J5" s="4">
+        <v>3.5959999999999998E-3</v>
+      </c>
+      <c r="K5" s="4">
+        <v>3.9950000000000003E-3</v>
+      </c>
+      <c r="L5" s="4">
+        <v>3.5959999999999998E-3</v>
+      </c>
+      <c r="M5" s="4">
+        <v>1.598E-3</v>
+      </c>
+      <c r="N5" s="4">
+        <v>1.598E-3</v>
+      </c>
+      <c r="O5" s="4">
+        <v>3.1960000000000001E-3</v>
+      </c>
+      <c r="P5" s="4">
+        <v>3.1960000000000001E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>42736</v>
       </c>
@@ -616,8 +2360,38 @@
       <c r="E6">
         <v>4.1840000000000002E-3</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G6" s="3">
+        <v>42826</v>
+      </c>
+      <c r="H6" s="5">
+        <v>1</v>
+      </c>
+      <c r="I6" s="4">
+        <v>6.2059999999999997E-3</v>
+      </c>
+      <c r="J6" s="4">
+        <v>2.2160000000000001E-3</v>
+      </c>
+      <c r="K6" s="4">
+        <v>1.7730000000000001E-3</v>
+      </c>
+      <c r="L6" s="4">
+        <v>2.66E-3</v>
+      </c>
+      <c r="M6" s="4">
+        <v>2.66E-3</v>
+      </c>
+      <c r="N6" s="4">
+        <v>3.5460000000000001E-3</v>
+      </c>
+      <c r="O6" s="4">
+        <v>3.1029999999999999E-3</v>
+      </c>
+      <c r="P6" s="4">
+        <v>3.1029999999999999E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>42736</v>
       </c>
@@ -633,8 +2407,38 @@
       <c r="E7">
         <v>1.395E-3</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G7" s="3">
+        <v>42856</v>
+      </c>
+      <c r="H7" s="5">
+        <v>1</v>
+      </c>
+      <c r="I7" s="4">
+        <v>4.6360000000000004E-3</v>
+      </c>
+      <c r="J7" s="4">
+        <v>4.6360000000000004E-3</v>
+      </c>
+      <c r="K7" s="4">
+        <v>2.898E-3</v>
+      </c>
+      <c r="L7" s="4">
+        <v>2.898E-3</v>
+      </c>
+      <c r="M7" s="4">
+        <v>3.1870000000000002E-3</v>
+      </c>
+      <c r="N7" s="4">
+        <v>4.0569999999999998E-3</v>
+      </c>
+      <c r="O7" s="4">
+        <v>1.449E-3</v>
+      </c>
+      <c r="P7" s="4">
+        <v>2.6080000000000001E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>42736</v>
       </c>
@@ -650,8 +2454,38 @@
       <c r="E8">
         <v>4.1840000000000002E-3</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G8" s="3">
+        <v>42887</v>
+      </c>
+      <c r="H8" s="5">
+        <v>1</v>
+      </c>
+      <c r="I8" s="4">
+        <v>4.9389999999999998E-3</v>
+      </c>
+      <c r="J8" s="4">
+        <v>3.9509999999999997E-3</v>
+      </c>
+      <c r="K8" s="4">
+        <v>4.2810000000000001E-3</v>
+      </c>
+      <c r="L8" s="4">
+        <v>2.9629999999999999E-3</v>
+      </c>
+      <c r="M8" s="4">
+        <v>3.9509999999999997E-3</v>
+      </c>
+      <c r="N8" s="4">
+        <v>3.6219999999999998E-3</v>
+      </c>
+      <c r="O8" s="4">
+        <v>2.3050000000000002E-3</v>
+      </c>
+      <c r="P8" s="4">
+        <v>1.317E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>42736</v>
       </c>
@@ -667,8 +2501,38 @@
       <c r="E9">
         <v>1.395E-3</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G9" s="3">
+        <v>42917</v>
+      </c>
+      <c r="H9" s="5">
+        <v>1</v>
+      </c>
+      <c r="I9" s="4">
+        <v>5.3299999999999997E-3</v>
+      </c>
+      <c r="J9" s="4">
+        <v>3.4650000000000002E-3</v>
+      </c>
+      <c r="K9" s="4">
+        <v>2.3990000000000001E-3</v>
+      </c>
+      <c r="L9" s="4">
+        <v>2.9320000000000001E-3</v>
+      </c>
+      <c r="M9" s="4">
+        <v>2.1320000000000002E-3</v>
+      </c>
+      <c r="N9" s="4">
+        <v>3.1979999999999999E-3</v>
+      </c>
+      <c r="O9" s="4">
+        <v>1.0660000000000001E-3</v>
+      </c>
+      <c r="P9" s="4">
+        <v>1.866E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>42736</v>
       </c>
@@ -684,8 +2548,38 @@
       <c r="E10">
         <v>1.395E-3</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G10" s="3">
+        <v>42948</v>
+      </c>
+      <c r="H10" s="5">
+        <v>1</v>
+      </c>
+      <c r="I10" s="4">
+        <v>6.9020000000000001E-3</v>
+      </c>
+      <c r="J10" s="4">
+        <v>3.4510000000000001E-3</v>
+      </c>
+      <c r="K10" s="4">
+        <v>2.7109999999999999E-3</v>
+      </c>
+      <c r="L10" s="4">
+        <v>3.4510000000000001E-3</v>
+      </c>
+      <c r="M10" s="4">
+        <v>5.176E-3</v>
+      </c>
+      <c r="N10" s="4">
+        <v>2.9580000000000001E-3</v>
+      </c>
+      <c r="O10" s="4">
+        <v>2.7109999999999999E-3</v>
+      </c>
+      <c r="P10" s="4">
+        <v>1.4790000000000001E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>42767</v>
       </c>
@@ -701,8 +2595,38 @@
       <c r="E11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G11" s="3">
+        <v>42979</v>
+      </c>
+      <c r="H11" s="5">
+        <v>1</v>
+      </c>
+      <c r="I11" s="4">
+        <v>6.9930000000000001E-3</v>
+      </c>
+      <c r="J11" s="4">
+        <v>5.4949999999999999E-3</v>
+      </c>
+      <c r="K11" s="4">
+        <v>2.7469999999999999E-3</v>
+      </c>
+      <c r="L11" s="4">
+        <v>4.496E-3</v>
+      </c>
+      <c r="M11" s="4">
+        <v>2.248E-3</v>
+      </c>
+      <c r="N11" s="4">
+        <v>2.248E-3</v>
+      </c>
+      <c r="O11" s="4">
+        <v>2.4979999999999998E-3</v>
+      </c>
+      <c r="P11" s="4">
+        <v>2.7469999999999999E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>42767</v>
       </c>
@@ -719,7 +2643,7 @@
         <v>1.843E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>42767</v>
       </c>
@@ -736,7 +2660,7 @@
         <v>3.0709999999999999E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>42767</v>
       </c>
@@ -753,7 +2677,7 @@
         <v>1.2290000000000001E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>42767</v>
       </c>
@@ -770,7 +2694,7 @@
         <v>4.3E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>42767</v>
       </c>
@@ -1910,9 +3834,21 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting pivot="1" sqref="I3:P11">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>